<commit_message>
big commit lots of stuff changed
</commit_message>
<xml_diff>
--- a/data/stats/supp_tables/fallcover-cc-anova.xlsx
+++ b/data/stats/supp_tables/fallcover-cc-anova.xlsx
@@ -11,6 +11,77 @@
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="22">
+  <si>
+    <t>model term</t>
+  </si>
+  <si>
+    <t>df1</t>
+  </si>
+  <si>
+    <t>df2</t>
+  </si>
+  <si>
+    <t>F.ratio</t>
+  </si>
+  <si>
+    <t>Chisq</t>
+  </si>
+  <si>
+    <t>p.value</t>
+  </si>
+  <si>
+    <t>till_id</t>
+  </si>
+  <si>
+    <t>Inf</t>
+  </si>
+  <si>
+    <t>cctrt_id</t>
+  </si>
+  <si>
+    <t>straw_id</t>
+  </si>
+  <si>
+    <t>weayear</t>
+  </si>
+  <si>
+    <t>till_id:cctrt_id</t>
+  </si>
+  <si>
+    <t>till_id:straw_id</t>
+  </si>
+  <si>
+    <t>till_id:weayear</t>
+  </si>
+  <si>
+    <t>cctrt_id:straw_id</t>
+  </si>
+  <si>
+    <t>cctrt_id:weayear</t>
+  </si>
+  <si>
+    <t>straw_id:weayear</t>
+  </si>
+  <si>
+    <t>till_id:cctrt_id:straw_id</t>
+  </si>
+  <si>
+    <t>till_id:cctrt_id:weayear</t>
+  </si>
+  <si>
+    <t>till_id:straw_id:weayear</t>
+  </si>
+  <si>
+    <t>cctrt_id:straw_id:weayear</t>
+  </si>
+  <si>
+    <t>till_id:cctrt_id:straw_id:weayear</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -354,51 +425,35 @@
   <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>model term</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>df1</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>df2</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>F.ratio</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Chisq</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>p.value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>till_id</t>
-        </is>
+    <row r="1" spans="1:6" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>6</v>
       </c>
       <c r="B2">
         <v>2</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
+      <c r="C2" t="s">
+        <v>7</v>
       </c>
       <c r="D2">
         <v>1.33</v>
@@ -407,22 +462,18 @@
         <v>2.66</v>
       </c>
       <c r="F2">
-        <v>0.2645892429994832</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>cctrt_id</t>
-        </is>
+        <v>0.2645892163594145</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
+        <v>8</v>
       </c>
       <c r="B3">
         <v>4</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
+      <c r="C3" t="s">
+        <v>7</v>
       </c>
       <c r="D3">
         <v>254.747</v>
@@ -431,22 +482,18 @@
         <v>1018.988</v>
       </c>
       <c r="F3">
-        <v>2.740698627067196E-219</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>straw_id</t>
-        </is>
+        <v>2.740697076453002E-219</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>9</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
+      <c r="C4" t="s">
+        <v>7</v>
       </c>
       <c r="D4">
         <v>2.662</v>
@@ -455,22 +502,18 @@
         <v>2.662</v>
       </c>
       <c r="F4">
-        <v>0.1027749986989869</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>weayear</t>
-        </is>
+        <v>0.1027750071055079</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
+        <v>10</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
+      <c r="C5" t="s">
+        <v>7</v>
       </c>
       <c r="D5">
         <v>221.23</v>
@@ -479,22 +522,18 @@
         <v>221.23</v>
       </c>
       <c r="F5">
-        <v>4.877026871664119E-50</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>till_id:cctrt_id</t>
-        </is>
+        <v>4.877029839105276E-50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>11</v>
       </c>
       <c r="B6">
         <v>8</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
+      <c r="C6" t="s">
+        <v>7</v>
       </c>
       <c r="D6">
         <v>5.593</v>
@@ -503,22 +542,18 @@
         <v>44.744</v>
       </c>
       <c r="F6">
-        <v>4.114191462409115E-07</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>till_id:straw_id</t>
-        </is>
+        <v>4.114191421062665E-07</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" t="s">
+        <v>12</v>
       </c>
       <c r="B7">
         <v>2</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
+      <c r="C7" t="s">
+        <v>7</v>
       </c>
       <c r="D7">
         <v>1.388</v>
@@ -527,22 +562,18 @@
         <v>2.776</v>
       </c>
       <c r="F7">
-        <v>0.2496396067753656</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>till_id:weayear</t>
-        </is>
+        <v>0.2496396176045122</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" t="s">
+        <v>13</v>
       </c>
       <c r="B8">
         <v>2</v>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
+      <c r="C8" t="s">
+        <v>7</v>
       </c>
       <c r="D8">
         <v>2.576</v>
@@ -551,22 +582,18 @@
         <v>5.152</v>
       </c>
       <c r="F8">
-        <v>0.07604249615264</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>cctrt_id:straw_id</t>
-        </is>
+        <v>0.07604249637818132</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" t="s">
+        <v>14</v>
       </c>
       <c r="B9">
         <v>4</v>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
+      <c r="C9" t="s">
+        <v>7</v>
       </c>
       <c r="D9">
         <v>2.058</v>
@@ -575,22 +602,18 @@
         <v>8.231999999999999</v>
       </c>
       <c r="F9">
-        <v>0.08349072992330604</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>cctrt_id:weayear</t>
-        </is>
+        <v>0.08349072284228033</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" t="s">
+        <v>15</v>
       </c>
       <c r="B10">
         <v>4</v>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
+      <c r="C10" t="s">
+        <v>7</v>
       </c>
       <c r="D10">
         <v>108.812</v>
@@ -599,22 +622,18 @@
         <v>435.248</v>
       </c>
       <c r="F10">
-        <v>6.705252052934674E-93</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>straw_id:weayear</t>
-        </is>
+        <v>6.705249270325326E-93</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" t="s">
+        <v>16</v>
       </c>
       <c r="B11">
         <v>1</v>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
+      <c r="C11" t="s">
+        <v>7</v>
       </c>
       <c r="D11">
         <v>4.376</v>
@@ -623,22 +642,18 @@
         <v>4.376</v>
       </c>
       <c r="F11">
-        <v>0.03644654436681943</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>till_id:cctrt_id:straw_id</t>
-        </is>
+        <v>0.03644654340608012</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" t="s">
+        <v>17</v>
       </c>
       <c r="B12">
         <v>8</v>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
+      <c r="C12" t="s">
+        <v>7</v>
       </c>
       <c r="D12">
         <v>0.849</v>
@@ -647,22 +662,18 @@
         <v>6.792</v>
       </c>
       <c r="F12">
-        <v>0.5591096336815535</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>till_id:cctrt_id:weayear</t>
-        </is>
+        <v>0.5591096237079554</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" t="s">
+        <v>18</v>
       </c>
       <c r="B13">
         <v>8</v>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
+      <c r="C13" t="s">
+        <v>7</v>
       </c>
       <c r="D13">
         <v>7.107</v>
@@ -671,22 +682,18 @@
         <v>56.856</v>
       </c>
       <c r="F13">
-        <v>1.92260348034585E-09</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>till_id:straw_id:weayear</t>
-        </is>
+        <v>1.922603731099829E-09</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" t="s">
+        <v>19</v>
       </c>
       <c r="B14">
         <v>2</v>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
+      <c r="C14" t="s">
+        <v>7</v>
       </c>
       <c r="D14">
         <v>2.368</v>
@@ -695,22 +702,18 @@
         <v>4.736</v>
       </c>
       <c r="F14">
-        <v>0.09368265645391015</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>cctrt_id:straw_id:weayear</t>
-        </is>
+        <v>0.09368266336737113</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" t="s">
+        <v>20</v>
       </c>
       <c r="B15">
         <v>4</v>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
+      <c r="C15" t="s">
+        <v>7</v>
       </c>
       <c r="D15">
         <v>2.187</v>
@@ -719,22 +722,18 @@
         <v>8.747999999999999</v>
       </c>
       <c r="F15">
-        <v>0.06770877588056823</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>till_id:cctrt_id:straw_id:weayear</t>
-        </is>
+        <v>0.06770877382334257</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" t="s">
+        <v>21</v>
       </c>
       <c r="B16">
         <v>8</v>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Inf</t>
-        </is>
+      <c r="C16" t="s">
+        <v>7</v>
       </c>
       <c r="D16">
         <v>1.653</v>
@@ -743,7 +742,7 @@
         <v>13.224</v>
       </c>
       <c r="F16">
-        <v>0.1043577389722224</v>
+        <v>0.1043577298091089</v>
       </c>
     </row>
   </sheetData>

</xml_diff>